<commit_message>
updated readme with more explanations and better output processing
</commit_message>
<xml_diff>
--- a/inst/toy_ctdata.xlsx
+++ b/inst/toy_ctdata.xlsx
@@ -831,7 +831,7 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
@@ -843,12 +843,10 @@
         <v>30</v>
       </c>
       <c r="F30" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="G30" s="1" t="n">
-        <v>18</v>
-      </c>
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
@@ -876,7 +874,7 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
@@ -897,7 +895,7 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>

</xml_diff>